<commit_message>
Number of cycles for scra14 corrected again
</commit_message>
<xml_diff>
--- a/analysis/derived_data/FT_STA-stats.xlsx
+++ b/analysis/derived_data/FT_STA-stats.xlsx
@@ -1459,16 +1459,16 @@
         <v>0</v>
       </c>
       <c r="D2">
-        <v>476</v>
+        <v>560</v>
       </c>
       <c r="E2">
-        <v>201.5</v>
+        <v>222.5</v>
       </c>
       <c r="F2">
         <v>165</v>
       </c>
       <c r="G2">
-        <v>214.8283035356375</v>
+        <v>244.6630335788388</v>
       </c>
       <c r="H2">
         <v>16</v>
@@ -6501,16 +6501,16 @@
         <v>0</v>
       </c>
       <c r="E3">
-        <v>476</v>
+        <v>560</v>
       </c>
       <c r="F3">
-        <v>284.8888888888889</v>
+        <v>322.2222222222222</v>
       </c>
       <c r="G3">
         <v>330</v>
       </c>
       <c r="H3">
-        <v>221.8245052087598</v>
+        <v>259.2671295101723</v>
       </c>
       <c r="I3">
         <v>9</v>
@@ -17206,7 +17206,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>476</v>
+        <v>560</v>
       </c>
       <c r="C4">
         <v>4</v>
@@ -30158,7 +30158,7 @@
         </is>
       </c>
       <c r="B8">
-        <v>476</v>
+        <v>560</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -47810,7 +47810,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>476</v>
+        <v>560</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -60862,7 +60862,7 @@
         </is>
       </c>
       <c r="B8">
-        <v>476</v>
+        <v>560</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>

</xml_diff>